<commit_message>
Chamol PO: set requisitioner to Woodlite International, remove PO number
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoEh7Mj6ZxttHm1PyDH2Zo
</commit_message>
<xml_diff>
--- a/outputs/Woodlite_PO_Chamol.xlsx
+++ b/outputs/Woodlite_PO_Chamol.xlsx
@@ -4802,7 +4802,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{880B0EBD-FC8B-4B4F-BCDD-2A683C677CDA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE51FBCB-DA33-4BF2-B702-1590597CB428}">
   <dimension ref="A2:G106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4847,11 +4847,7 @@
           <t xml:space="preserve">DATE: 12-10-2026</t>
         </is>
       </c>
-      <c r="E6" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PO NUMBER: [TO BE ASSIGNED]</t>
-        </is>
-      </c>
+      <c r="E6" s="52"/>
     </row>
     <row r="7" spans="1:7" s="5" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A7" s="8"/>
@@ -4963,7 +4959,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Amadi Kinikanwo</t>
+          <t xml:space="preserve">Woodlite International</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -5366,8 +5362,8 @@
     <mergeCell ref="A45:B45"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{FC4ECE9B-F79A-45F1-9435-E7D46DD8DD70}"/>
-    <hyperlink ref="A40" r:id="rId2" xr:uid="{61651D3A-D850-4904-BA22-5D5196C43D97}"/>
+    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{0BAFD52A-098F-4F9F-8F1C-3DBA7DAA27DE}"/>
+    <hyperlink ref="A40" r:id="rId2" xr:uid="{38CC7457-D78D-416B-8ECB-1D832B416D01}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="1.1299999999999999" bottom="0.75" header="0.35" footer="0.3"/>
   <pageSetup scale="78" orientation="portrait" r:id="rId3"/>

</xml_diff>

<commit_message>
Chamol PO: add Woodlite seal to the quotation page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoEh7Mj6ZxttHm1PyDH2Zo
</commit_message>
<xml_diff>
--- a/outputs/Woodlite_PO_Chamol.xlsx
+++ b/outputs/Woodlite_PO_Chamol.xlsx
@@ -1492,6 +1492,39 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>981075</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2038350" cy="1285875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Woodlite Seal"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2038350" cy="1285875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4802,7 +4835,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE51FBCB-DA33-4BF2-B702-1590597CB428}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E54B1D4B-4C58-4667-9914-8F2E79182167}">
   <dimension ref="A2:G106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5362,8 +5395,8 @@
     <mergeCell ref="A45:B45"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{0BAFD52A-098F-4F9F-8F1C-3DBA7DAA27DE}"/>
-    <hyperlink ref="A40" r:id="rId2" xr:uid="{38CC7457-D78D-416B-8ECB-1D832B416D01}"/>
+    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{D4B1BD7B-57A0-42A5-A10C-B79EDF39AFA3}"/>
+    <hyperlink ref="A40" r:id="rId2" xr:uid="{63C5CC56-CBA0-4C68-A50B-CB76523505EE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="1.1299999999999999" bottom="0.75" header="0.35" footer="0.3"/>
   <pageSetup scale="78" orientation="portrait" r:id="rId3"/>

</xml_diff>

<commit_message>
Chamol PO: move seal on quotation page to the left
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoEh7Mj6ZxttHm1PyDH2Zo
</commit_message>
<xml_diff>
--- a/outputs/Woodlite_PO_Chamol.xlsx
+++ b/outputs/Woodlite_PO_Chamol.xlsx
@@ -1494,8 +1494,8 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>981075</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
       <xdr:row>95</xdr:row>
       <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
@@ -4835,7 +4835,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E54B1D4B-4C58-4667-9914-8F2E79182167}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385F0503-BD0D-401C-8C6C-42B65B8A1060}">
   <dimension ref="A2:G106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5395,8 +5395,8 @@
     <mergeCell ref="A45:B45"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{D4B1BD7B-57A0-42A5-A10C-B79EDF39AFA3}"/>
-    <hyperlink ref="A40" r:id="rId2" xr:uid="{63C5CC56-CBA0-4C68-A50B-CB76523505EE}"/>
+    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{E243124E-42BE-43E6-9CEF-D3D5C9C378A5}"/>
+    <hyperlink ref="A40" r:id="rId2" xr:uid="{FFB5AB89-7FD8-4DFC-A859-EAC87EE87FB5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="1.1299999999999999" bottom="0.75" header="0.35" footer="0.3"/>
   <pageSetup scale="78" orientation="portrait" r:id="rId3"/>

</xml_diff>